<commit_message>
Daily slate 2026-05-19 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-17.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-17.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
         <v>11</v>
       </c>
       <c r="G4" t="n">
-        <v>50</v>
+        <v>54.2</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F5" t="n">
         <v>17</v>
       </c>
       <c r="G5" t="n">
-        <v>51.4</v>
+        <v>54.1</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
         <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G6" t="n">
-        <v>56</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" t="n">
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G7" t="n">
-        <v>38.7</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="8">
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5716</v>
+        <v>5705</v>
       </c>
       <c r="E8" t="n">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="F8" t="n">
-        <v>4833</v>
+        <v>4824</v>
       </c>
       <c r="G8" t="n">
         <v>15.4</v>
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>602</v>
+        <v>635</v>
       </c>
       <c r="E10" t="n">
-        <v>406</v>
+        <v>430</v>
       </c>
       <c r="F10" t="n">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="G10" t="n">
-        <v>67.40000000000001</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>425</v>
+        <v>442</v>
       </c>
       <c r="E11" t="n">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="F11" t="n">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="G11" t="n">
-        <v>62.4</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E12" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F12" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G12" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E13" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F13" t="n">
         <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>57.3</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="E14" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F14" t="n">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="G14" t="n">
-        <v>24.4</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="E15" t="n">
         <v>68</v>
       </c>
       <c r="F15" t="n">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G15" t="n">
-        <v>18.3</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E16" t="n">
         <v>32</v>
       </c>
       <c r="F16" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G16" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="17">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2545</v>
+        <v>2735</v>
       </c>
       <c r="E17" t="n">
-        <v>609</v>
+        <v>653</v>
       </c>
       <c r="F17" t="n">
-        <v>1936</v>
+        <v>2082</v>
       </c>
       <c r="G17" t="n">
         <v>23.9</v>
@@ -1166,10 +1166,10 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="Z2" t="n">
         <v>50</v>
@@ -1421,10 +1421,10 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>12.8</v>
+        <v>12.3</v>
       </c>
       <c r="Y5" t="n">
-        <v>733</v>
+        <v>716</v>
       </c>
       <c r="Z5" t="n">
         <v>100</v>
@@ -1552,52 +1552,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>67.40000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="C7" t="n">
-        <v>602</v>
+        <v>635</v>
       </c>
       <c r="D7" t="n">
-        <v>62.4</v>
+        <v>62.2</v>
       </c>
       <c r="E7" t="n">
-        <v>425</v>
+        <v>442</v>
       </c>
       <c r="F7" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
       <c r="G7" t="n">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H7" t="n">
-        <v>57.3</v>
+        <v>57.6</v>
       </c>
       <c r="I7" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J7" t="n">
-        <v>24.4</v>
+        <v>23.9</v>
       </c>
       <c r="K7" t="n">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="L7" t="n">
-        <v>18.3</v>
+        <v>18.1</v>
       </c>
       <c r="M7" t="n">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="N7" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
       <c r="O7" t="n">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="P7" t="n">
         <v>23.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>2545</v>
+        <v>2735</v>
       </c>
       <c r="R7" t="n">
         <v>34.8</v>
@@ -1606,22 +1606,22 @@
         <v>46</v>
       </c>
       <c r="T7" t="n">
-        <v>50</v>
+        <v>54.2</v>
       </c>
       <c r="U7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="V7" t="n">
-        <v>56</v>
+        <v>51.9</v>
       </c>
       <c r="W7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="X7" t="n">
         <v>15.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>5716</v>
+        <v>5705</v>
       </c>
       <c r="Z7" t="n">
         <v>62.6</v>
@@ -1630,16 +1630,16 @@
         <v>214</v>
       </c>
       <c r="AB7" t="n">
-        <v>51.4</v>
+        <v>54.1</v>
       </c>
       <c r="AC7" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AD7" t="n">
-        <v>38.7</v>
+        <v>37.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AF7" t="n">
         <v>61.5</v>

</xml_diff>